<commit_message>
Painel web ao vivo Lula x Flávio Bolsonaro e planilha sem dados fictícios
- painel-ao-vivo/: página com placar, probabilidade de vitória e gráficos,
  atualizando a cada 30 s a partir do arquivo EA20 do TSE; servidor local
  (Python ou PowerShell) repassa o JSON do TSE e evita o bloqueio CORS
- planilha: remove a demonstração e cadastra Lula (13) e Flávio Bolsonaro (22)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rnp9d59qD4FX5kiUK6SDfo
</commit_message>
<xml_diff>
--- a/apuracao-2turno/apuracao_2turno.xlsx
+++ b/apuracao-2turno/apuracao_2turno.xlsx
@@ -357,7 +357,7 @@
           <idx val="0"/>
           <order val="0"/>
           <tx>
-            <v>Candidato 1</v>
+            <v>Lula (13)</v>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
@@ -398,7 +398,7 @@
           <idx val="1"/>
           <order val="1"/>
           <tx>
-            <v>Candidato 2</v>
+            <v>Flávio Bolsonaro (22)</v>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
@@ -533,7 +533,7 @@
           <idx val="0"/>
           <order val="0"/>
           <tx>
-            <v>Candidato 1</v>
+            <v>Lula (13)</v>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
@@ -574,7 +574,7 @@
           <idx val="1"/>
           <order val="1"/>
           <tx>
-            <v>Candidato 2</v>
+            <v>Flávio Bolsonaro (22)</v>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
@@ -1768,7 +1768,7 @@
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Ajuste de tendência p/ candidato 1 (p.p.)</t>
+          <t>Ajuste de tendência p/ Lula (p.p.)</t>
         </is>
       </c>
       <c r="B17" s="29" t="n">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="C17" s="25" t="inlineStr">
         <is>
-          <t>Ex.: +0,02 se você espera que as urnas restantes favoreçam o cand. 1 em 2 p.p.</t>
+          <t>Ex.: +0,02 se você espera que as urnas restantes favoreçam Lula em 2 p.p. (negativo favorece Flávio)</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="B22" s="25" t="inlineStr">
         <is>
-          <t>A planilha vem com DADOS DE DEMONSTRAÇÃO (candidatos fictícios). Antes de conectar, siga a aba 'Como usar'. A probabilidade é uma estimativa estatística — o resultado oficial é sempre o do TSE.</t>
+          <t>Lula (13) e Flávio Bolsonaro (22) já estão cadastrados; os votos chegam pela conexão (aba 'Como usar'). Para acompanhar sem configurar nada, use o painel web da pasta painel-ao-vivo. A probabilidade é uma estimativa; o resultado oficial é sempre o do TSE.</t>
         </is>
       </c>
     </row>
@@ -1926,20 +1926,20 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CANDIDATO A (DEMO)</t>
+          <t>LULA</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>PART-A</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>54862312</v>
+        <v>0</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1972,16 +1972,16 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>CANDIDATO B (DEMO)</t>
+          <t>FLÁVIO BOLSONARO</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>PART-B</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>55925781</v>
+        <v>0</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -1990,7 +1990,7 @@
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -2050,11 +2050,7 @@
           <t>dt</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" s="31" t="inlineStr">
         <is>
           <t>Data da totalização</t>
@@ -2067,11 +2063,7 @@
           <t>ht</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>19:29:00</t>
-        </is>
-      </c>
+      <c r="B8" t="inlineStr"/>
       <c r="C8" s="31" t="inlineStr">
         <is>
           <t>Hora da totalização</t>
@@ -2086,7 +2078,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>p</t>
+          <t>n</t>
         </is>
       </c>
       <c r="C9" s="31" t="inlineStr">
@@ -2137,7 +2129,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>n</t>
         </is>
       </c>
       <c r="C12" s="31" t="inlineStr">
@@ -2153,7 +2145,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>472075</v>
+        <v>0</v>
       </c>
       <c r="C13" s="31" t="inlineStr">
         <is>
@@ -2168,7 +2160,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>443750</v>
+        <v>0</v>
       </c>
       <c r="C14" s="31" t="inlineStr">
         <is>
@@ -2183,7 +2175,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>156454011</v>
+        <v>0</v>
       </c>
       <c r="C15" s="31" t="inlineStr">
         <is>
@@ -2198,7 +2190,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>147066770</v>
+        <v>0</v>
       </c>
       <c r="C16" s="31" t="inlineStr">
         <is>
@@ -2213,7 +2205,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>146846170</v>
+        <v>0</v>
       </c>
       <c r="C17" s="31" t="inlineStr">
         <is>
@@ -2228,7 +2220,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>116008474</v>
+        <v>0</v>
       </c>
       <c r="C18" s="31" t="inlineStr">
         <is>
@@ -2243,7 +2235,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>30837696</v>
+        <v>0</v>
       </c>
       <c r="C19" s="31" t="inlineStr">
         <is>
@@ -2258,7 +2250,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>116008474</v>
+        <v>0</v>
       </c>
       <c r="C20" s="31" t="inlineStr">
         <is>
@@ -2273,7 +2265,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>110788093</v>
+        <v>0</v>
       </c>
       <c r="C21" s="31" t="inlineStr">
         <is>
@@ -2288,7 +2280,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1827133</v>
+        <v>0</v>
       </c>
       <c r="C22" s="31" t="inlineStr">
         <is>
@@ -2303,7 +2295,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3393248</v>
+        <v>0</v>
       </c>
       <c r="C23" s="31" t="inlineStr">
         <is>
@@ -2458,12 +2450,12 @@
       </c>
       <c r="P1" s="32" t="inlineStr">
         <is>
-          <t>% válidos cand.1</t>
+          <t>% válidos Lula</t>
         </is>
       </c>
       <c r="Q1" s="32" t="inlineStr">
         <is>
-          <t>% válidos cand.2</t>
+          <t>% válidos Flávio</t>
         </is>
       </c>
       <c r="R1" s="32" t="inlineStr">
@@ -2473,61 +2465,31 @@
       </c>
       <c r="S1" s="32" t="inlineStr">
         <is>
-          <t>Fatia que o cand.1 precisa</t>
+          <t>Fatia que Lula precisa</t>
         </is>
       </c>
       <c r="T1" s="32" t="inlineStr">
         <is>
-          <t>Prob. cand.1</t>
+          <t>Prob. Lula</t>
         </is>
       </c>
       <c r="U1" s="32" t="inlineStr">
         <is>
-          <t>Prob. cand.2</t>
+          <t>Prob. Flávio</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>17:05:00</t>
-        </is>
-      </c>
-      <c r="C2" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D2" s="33" t="n">
-        <v>1888</v>
-      </c>
-      <c r="E2" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F2" s="33" t="n">
-        <v>625816</v>
-      </c>
-      <c r="G2" s="33" t="n">
-        <v>624877</v>
-      </c>
-      <c r="H2" s="33" t="n">
-        <v>493653</v>
-      </c>
-      <c r="I2" s="33" t="n">
-        <v>493653</v>
-      </c>
-      <c r="J2" s="33" t="n">
-        <v>471439</v>
-      </c>
-      <c r="K2" s="33" t="n">
-        <v>252199</v>
-      </c>
-      <c r="L2" s="33" t="n">
-        <v>219240</v>
-      </c>
+      <c r="C2" s="33" t="n"/>
+      <c r="D2" s="33" t="n"/>
+      <c r="E2" s="33" t="n"/>
+      <c r="F2" s="33" t="n"/>
+      <c r="G2" s="33" t="n"/>
+      <c r="H2" s="33" t="n"/>
+      <c r="I2" s="33" t="n"/>
+      <c r="J2" s="33" t="n"/>
+      <c r="K2" s="33" t="n"/>
+      <c r="L2" s="33" t="n"/>
       <c r="N2" s="34">
         <f>IF($A2="",NA(),IF(C2&gt;0,D2/C2,0))</f>
         <v/>
@@ -2562,46 +2524,16 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>17:11:00</t>
-        </is>
-      </c>
-      <c r="C3" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D3" s="33" t="n">
-        <v>4721</v>
-      </c>
-      <c r="E3" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F3" s="33" t="n">
-        <v>1564540</v>
-      </c>
-      <c r="G3" s="33" t="n">
-        <v>1562193</v>
-      </c>
-      <c r="H3" s="33" t="n">
-        <v>1234132</v>
-      </c>
-      <c r="I3" s="33" t="n">
-        <v>1234132</v>
-      </c>
-      <c r="J3" s="33" t="n">
-        <v>1178596</v>
-      </c>
-      <c r="K3" s="33" t="n">
-        <v>630389</v>
-      </c>
-      <c r="L3" s="33" t="n">
-        <v>548207</v>
-      </c>
+      <c r="C3" s="33" t="n"/>
+      <c r="D3" s="33" t="n"/>
+      <c r="E3" s="33" t="n"/>
+      <c r="F3" s="33" t="n"/>
+      <c r="G3" s="33" t="n"/>
+      <c r="H3" s="33" t="n"/>
+      <c r="I3" s="33" t="n"/>
+      <c r="J3" s="33" t="n"/>
+      <c r="K3" s="33" t="n"/>
+      <c r="L3" s="33" t="n"/>
       <c r="N3" s="34">
         <f>IF($A3="",NA(),IF(C3&gt;0,D3/C3,0))</f>
         <v/>
@@ -2636,46 +2568,16 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>17:17:00</t>
-        </is>
-      </c>
-      <c r="C4" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D4" s="33" t="n">
-        <v>9442</v>
-      </c>
-      <c r="E4" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F4" s="33" t="n">
-        <v>3129080</v>
-      </c>
-      <c r="G4" s="33" t="n">
-        <v>3124386</v>
-      </c>
-      <c r="H4" s="33" t="n">
-        <v>2468265</v>
-      </c>
-      <c r="I4" s="33" t="n">
-        <v>2468265</v>
-      </c>
-      <c r="J4" s="33" t="n">
-        <v>2357193</v>
-      </c>
-      <c r="K4" s="33" t="n">
-        <v>1260336</v>
-      </c>
-      <c r="L4" s="33" t="n">
-        <v>1096857</v>
-      </c>
+      <c r="C4" s="33" t="n"/>
+      <c r="D4" s="33" t="n"/>
+      <c r="E4" s="33" t="n"/>
+      <c r="F4" s="33" t="n"/>
+      <c r="G4" s="33" t="n"/>
+      <c r="H4" s="33" t="n"/>
+      <c r="I4" s="33" t="n"/>
+      <c r="J4" s="33" t="n"/>
+      <c r="K4" s="33" t="n"/>
+      <c r="L4" s="33" t="n"/>
       <c r="N4" s="34">
         <f>IF($A4="",NA(),IF(C4&gt;0,D4/C4,0))</f>
         <v/>
@@ -2710,46 +2612,16 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>17:23:00</t>
-        </is>
-      </c>
-      <c r="C5" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D5" s="33" t="n">
-        <v>18883</v>
-      </c>
-      <c r="E5" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F5" s="33" t="n">
-        <v>6258160</v>
-      </c>
-      <c r="G5" s="33" t="n">
-        <v>6248773</v>
-      </c>
-      <c r="H5" s="33" t="n">
-        <v>4936531</v>
-      </c>
-      <c r="I5" s="33" t="n">
-        <v>4936531</v>
-      </c>
-      <c r="J5" s="33" t="n">
-        <v>4714387</v>
-      </c>
-      <c r="K5" s="33" t="n">
-        <v>2518571</v>
-      </c>
-      <c r="L5" s="33" t="n">
-        <v>2195816</v>
-      </c>
+      <c r="C5" s="33" t="n"/>
+      <c r="D5" s="33" t="n"/>
+      <c r="E5" s="33" t="n"/>
+      <c r="F5" s="33" t="n"/>
+      <c r="G5" s="33" t="n"/>
+      <c r="H5" s="33" t="n"/>
+      <c r="I5" s="33" t="n"/>
+      <c r="J5" s="33" t="n"/>
+      <c r="K5" s="33" t="n"/>
+      <c r="L5" s="33" t="n"/>
       <c r="N5" s="34">
         <f>IF($A5="",NA(),IF(C5&gt;0,D5/C5,0))</f>
         <v/>
@@ -2784,46 +2656,16 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>17:29:00</t>
-        </is>
-      </c>
-      <c r="C6" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D6" s="33" t="n">
-        <v>33045</v>
-      </c>
-      <c r="E6" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F6" s="33" t="n">
-        <v>10951781</v>
-      </c>
-      <c r="G6" s="33" t="n">
-        <v>10935353</v>
-      </c>
-      <c r="H6" s="33" t="n">
-        <v>8638929</v>
-      </c>
-      <c r="I6" s="33" t="n">
-        <v>8638929</v>
-      </c>
-      <c r="J6" s="33" t="n">
-        <v>8250177</v>
-      </c>
-      <c r="K6" s="33" t="n">
-        <v>4401071</v>
-      </c>
-      <c r="L6" s="33" t="n">
-        <v>3849106</v>
-      </c>
+      <c r="C6" s="33" t="n"/>
+      <c r="D6" s="33" t="n"/>
+      <c r="E6" s="33" t="n"/>
+      <c r="F6" s="33" t="n"/>
+      <c r="G6" s="33" t="n"/>
+      <c r="H6" s="33" t="n"/>
+      <c r="I6" s="33" t="n"/>
+      <c r="J6" s="33" t="n"/>
+      <c r="K6" s="33" t="n"/>
+      <c r="L6" s="33" t="n"/>
       <c r="N6" s="34">
         <f>IF($A6="",NA(),IF(C6&gt;0,D6/C6,0))</f>
         <v/>
@@ -2858,46 +2700,16 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>17:35:00</t>
-        </is>
-      </c>
-      <c r="C7" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D7" s="33" t="n">
-        <v>47208</v>
-      </c>
-      <c r="E7" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F7" s="33" t="n">
-        <v>15645401</v>
-      </c>
-      <c r="G7" s="33" t="n">
-        <v>15621933</v>
-      </c>
-      <c r="H7" s="33" t="n">
-        <v>12341327</v>
-      </c>
-      <c r="I7" s="33" t="n">
-        <v>12341327</v>
-      </c>
-      <c r="J7" s="33" t="n">
-        <v>11785967</v>
-      </c>
-      <c r="K7" s="33" t="n">
-        <v>6276993</v>
-      </c>
-      <c r="L7" s="33" t="n">
-        <v>5508974</v>
-      </c>
+      <c r="C7" s="33" t="n"/>
+      <c r="D7" s="33" t="n"/>
+      <c r="E7" s="33" t="n"/>
+      <c r="F7" s="33" t="n"/>
+      <c r="G7" s="33" t="n"/>
+      <c r="H7" s="33" t="n"/>
+      <c r="I7" s="33" t="n"/>
+      <c r="J7" s="33" t="n"/>
+      <c r="K7" s="33" t="n"/>
+      <c r="L7" s="33" t="n"/>
       <c r="N7" s="34">
         <f>IF($A7="",NA(),IF(C7&gt;0,D7/C7,0))</f>
         <v/>
@@ -2932,46 +2744,16 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>17:41:00</t>
-        </is>
-      </c>
-      <c r="C8" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D8" s="33" t="n">
-        <v>66090</v>
-      </c>
-      <c r="E8" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F8" s="33" t="n">
-        <v>21903562</v>
-      </c>
-      <c r="G8" s="33" t="n">
-        <v>21870707</v>
-      </c>
-      <c r="H8" s="33" t="n">
-        <v>17277859</v>
-      </c>
-      <c r="I8" s="33" t="n">
-        <v>17277859</v>
-      </c>
-      <c r="J8" s="33" t="n">
-        <v>16500355</v>
-      </c>
-      <c r="K8" s="33" t="n">
-        <v>8766929</v>
-      </c>
-      <c r="L8" s="33" t="n">
-        <v>7733426</v>
-      </c>
+      <c r="C8" s="33" t="n"/>
+      <c r="D8" s="33" t="n"/>
+      <c r="E8" s="33" t="n"/>
+      <c r="F8" s="33" t="n"/>
+      <c r="G8" s="33" t="n"/>
+      <c r="H8" s="33" t="n"/>
+      <c r="I8" s="33" t="n"/>
+      <c r="J8" s="33" t="n"/>
+      <c r="K8" s="33" t="n"/>
+      <c r="L8" s="33" t="n"/>
       <c r="N8" s="34">
         <f>IF($A8="",NA(),IF(C8&gt;0,D8/C8,0))</f>
         <v/>
@@ -3006,46 +2788,16 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>17:47:00</t>
-        </is>
-      </c>
-      <c r="C9" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D9" s="33" t="n">
-        <v>89694</v>
-      </c>
-      <c r="E9" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F9" s="33" t="n">
-        <v>29726262</v>
-      </c>
-      <c r="G9" s="33" t="n">
-        <v>29681673</v>
-      </c>
-      <c r="H9" s="33" t="n">
-        <v>23448522</v>
-      </c>
-      <c r="I9" s="33" t="n">
-        <v>23448522</v>
-      </c>
-      <c r="J9" s="33" t="n">
-        <v>22393339</v>
-      </c>
-      <c r="K9" s="33" t="n">
-        <v>11859647</v>
-      </c>
-      <c r="L9" s="33" t="n">
-        <v>10533692</v>
-      </c>
+      <c r="C9" s="33" t="n"/>
+      <c r="D9" s="33" t="n"/>
+      <c r="E9" s="33" t="n"/>
+      <c r="F9" s="33" t="n"/>
+      <c r="G9" s="33" t="n"/>
+      <c r="H9" s="33" t="n"/>
+      <c r="I9" s="33" t="n"/>
+      <c r="J9" s="33" t="n"/>
+      <c r="K9" s="33" t="n"/>
+      <c r="L9" s="33" t="n"/>
       <c r="N9" s="34">
         <f>IF($A9="",NA(),IF(C9&gt;0,D9/C9,0))</f>
         <v/>
@@ -3080,46 +2832,16 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>17:53:00</t>
-        </is>
-      </c>
-      <c r="C10" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D10" s="33" t="n">
-        <v>118019</v>
-      </c>
-      <c r="E10" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F10" s="33" t="n">
-        <v>39113503</v>
-      </c>
-      <c r="G10" s="33" t="n">
-        <v>39054833</v>
-      </c>
-      <c r="H10" s="33" t="n">
-        <v>30853318</v>
-      </c>
-      <c r="I10" s="33" t="n">
-        <v>30853318</v>
-      </c>
-      <c r="J10" s="33" t="n">
-        <v>29464919</v>
-      </c>
-      <c r="K10" s="33" t="n">
-        <v>15539757</v>
-      </c>
-      <c r="L10" s="33" t="n">
-        <v>13925162</v>
-      </c>
+      <c r="C10" s="33" t="n"/>
+      <c r="D10" s="33" t="n"/>
+      <c r="E10" s="33" t="n"/>
+      <c r="F10" s="33" t="n"/>
+      <c r="G10" s="33" t="n"/>
+      <c r="H10" s="33" t="n"/>
+      <c r="I10" s="33" t="n"/>
+      <c r="J10" s="33" t="n"/>
+      <c r="K10" s="33" t="n"/>
+      <c r="L10" s="33" t="n"/>
       <c r="N10" s="34">
         <f>IF($A10="",NA(),IF(C10&gt;0,D10/C10,0))</f>
         <v/>
@@ -3154,46 +2876,16 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>17:59:00</t>
-        </is>
-      </c>
-      <c r="C11" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D11" s="33" t="n">
-        <v>146343</v>
-      </c>
-      <c r="E11" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F11" s="33" t="n">
-        <v>48500743</v>
-      </c>
-      <c r="G11" s="33" t="n">
-        <v>48427992</v>
-      </c>
-      <c r="H11" s="33" t="n">
-        <v>38258114</v>
-      </c>
-      <c r="I11" s="33" t="n">
-        <v>38258114</v>
-      </c>
-      <c r="J11" s="33" t="n">
-        <v>36536499</v>
-      </c>
-      <c r="K11" s="33" t="n">
-        <v>19183616</v>
-      </c>
-      <c r="L11" s="33" t="n">
-        <v>17352883</v>
-      </c>
+      <c r="C11" s="33" t="n"/>
+      <c r="D11" s="33" t="n"/>
+      <c r="E11" s="33" t="n"/>
+      <c r="F11" s="33" t="n"/>
+      <c r="G11" s="33" t="n"/>
+      <c r="H11" s="33" t="n"/>
+      <c r="I11" s="33" t="n"/>
+      <c r="J11" s="33" t="n"/>
+      <c r="K11" s="33" t="n"/>
+      <c r="L11" s="33" t="n"/>
       <c r="N11" s="34">
         <f>IF($A11="",NA(),IF(C11&gt;0,D11/C11,0))</f>
         <v/>
@@ -3228,46 +2920,16 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>18:05:00</t>
-        </is>
-      </c>
-      <c r="C12" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D12" s="33" t="n">
-        <v>174668</v>
-      </c>
-      <c r="E12" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F12" s="33" t="n">
-        <v>57887984</v>
-      </c>
-      <c r="G12" s="33" t="n">
-        <v>57801152</v>
-      </c>
-      <c r="H12" s="33" t="n">
-        <v>45662910</v>
-      </c>
-      <c r="I12" s="33" t="n">
-        <v>45662910</v>
-      </c>
-      <c r="J12" s="33" t="n">
-        <v>43608079</v>
-      </c>
-      <c r="K12" s="33" t="n">
-        <v>22789210</v>
-      </c>
-      <c r="L12" s="33" t="n">
-        <v>20818869</v>
-      </c>
+      <c r="C12" s="33" t="n"/>
+      <c r="D12" s="33" t="n"/>
+      <c r="E12" s="33" t="n"/>
+      <c r="F12" s="33" t="n"/>
+      <c r="G12" s="33" t="n"/>
+      <c r="H12" s="33" t="n"/>
+      <c r="I12" s="33" t="n"/>
+      <c r="J12" s="33" t="n"/>
+      <c r="K12" s="33" t="n"/>
+      <c r="L12" s="33" t="n"/>
       <c r="N12" s="34">
         <f>IF($A12="",NA(),IF(C12&gt;0,D12/C12,0))</f>
         <v/>
@@ -3302,46 +2964,16 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>18:11:00</t>
-        </is>
-      </c>
-      <c r="C13" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D13" s="33" t="n">
-        <v>202992</v>
-      </c>
-      <c r="E13" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F13" s="33" t="n">
-        <v>67275225</v>
-      </c>
-      <c r="G13" s="33" t="n">
-        <v>67174312</v>
-      </c>
-      <c r="H13" s="33" t="n">
-        <v>53067706</v>
-      </c>
-      <c r="I13" s="33" t="n">
-        <v>53067706</v>
-      </c>
-      <c r="J13" s="33" t="n">
-        <v>50679659</v>
-      </c>
-      <c r="K13" s="33" t="n">
-        <v>26354799</v>
-      </c>
-      <c r="L13" s="33" t="n">
-        <v>24324860</v>
-      </c>
+      <c r="C13" s="33" t="n"/>
+      <c r="D13" s="33" t="n"/>
+      <c r="E13" s="33" t="n"/>
+      <c r="F13" s="33" t="n"/>
+      <c r="G13" s="33" t="n"/>
+      <c r="H13" s="33" t="n"/>
+      <c r="I13" s="33" t="n"/>
+      <c r="J13" s="33" t="n"/>
+      <c r="K13" s="33" t="n"/>
+      <c r="L13" s="33" t="n"/>
       <c r="N13" s="34">
         <f>IF($A13="",NA(),IF(C13&gt;0,D13/C13,0))</f>
         <v/>
@@ -3376,46 +3008,16 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>18:17:00</t>
-        </is>
-      </c>
-      <c r="C14" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D14" s="33" t="n">
-        <v>231317</v>
-      </c>
-      <c r="E14" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F14" s="33" t="n">
-        <v>76662465</v>
-      </c>
-      <c r="G14" s="33" t="n">
-        <v>76547471</v>
-      </c>
-      <c r="H14" s="33" t="n">
-        <v>60472502</v>
-      </c>
-      <c r="I14" s="33" t="n">
-        <v>60472502</v>
-      </c>
-      <c r="J14" s="33" t="n">
-        <v>57751239</v>
-      </c>
-      <c r="K14" s="33" t="n">
-        <v>29878849</v>
-      </c>
-      <c r="L14" s="33" t="n">
-        <v>27872390</v>
-      </c>
+      <c r="C14" s="33" t="n"/>
+      <c r="D14" s="33" t="n"/>
+      <c r="E14" s="33" t="n"/>
+      <c r="F14" s="33" t="n"/>
+      <c r="G14" s="33" t="n"/>
+      <c r="H14" s="33" t="n"/>
+      <c r="I14" s="33" t="n"/>
+      <c r="J14" s="33" t="n"/>
+      <c r="K14" s="33" t="n"/>
+      <c r="L14" s="33" t="n"/>
       <c r="N14" s="34">
         <f>IF($A14="",NA(),IF(C14&gt;0,D14/C14,0))</f>
         <v/>
@@ -3450,46 +3052,16 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>18:23:00</t>
-        </is>
-      </c>
-      <c r="C15" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D15" s="33" t="n">
-        <v>259641</v>
-      </c>
-      <c r="E15" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F15" s="33" t="n">
-        <v>86049706</v>
-      </c>
-      <c r="G15" s="33" t="n">
-        <v>85920631</v>
-      </c>
-      <c r="H15" s="33" t="n">
-        <v>67877298</v>
-      </c>
-      <c r="I15" s="33" t="n">
-        <v>67877298</v>
-      </c>
-      <c r="J15" s="33" t="n">
-        <v>64822820</v>
-      </c>
-      <c r="K15" s="33" t="n">
-        <v>33359978</v>
-      </c>
-      <c r="L15" s="33" t="n">
-        <v>31462842</v>
-      </c>
+      <c r="C15" s="33" t="n"/>
+      <c r="D15" s="33" t="n"/>
+      <c r="E15" s="33" t="n"/>
+      <c r="F15" s="33" t="n"/>
+      <c r="G15" s="33" t="n"/>
+      <c r="H15" s="33" t="n"/>
+      <c r="I15" s="33" t="n"/>
+      <c r="J15" s="33" t="n"/>
+      <c r="K15" s="33" t="n"/>
+      <c r="L15" s="33" t="n"/>
       <c r="N15" s="34">
         <f>IF($A15="",NA(),IF(C15&gt;0,D15/C15,0))</f>
         <v/>
@@ -3524,46 +3096,16 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>18:29:00</t>
-        </is>
-      </c>
-      <c r="C16" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D16" s="33" t="n">
-        <v>283245</v>
-      </c>
-      <c r="E16" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F16" s="33" t="n">
-        <v>93872407</v>
-      </c>
-      <c r="G16" s="33" t="n">
-        <v>93731598</v>
-      </c>
-      <c r="H16" s="33" t="n">
-        <v>74047962</v>
-      </c>
-      <c r="I16" s="33" t="n">
-        <v>74047962</v>
-      </c>
-      <c r="J16" s="33" t="n">
-        <v>70715804</v>
-      </c>
-      <c r="K16" s="33" t="n">
-        <v>36227220</v>
-      </c>
-      <c r="L16" s="33" t="n">
-        <v>34488584</v>
-      </c>
+      <c r="C16" s="33" t="n"/>
+      <c r="D16" s="33" t="n"/>
+      <c r="E16" s="33" t="n"/>
+      <c r="F16" s="33" t="n"/>
+      <c r="G16" s="33" t="n"/>
+      <c r="H16" s="33" t="n"/>
+      <c r="I16" s="33" t="n"/>
+      <c r="J16" s="33" t="n"/>
+      <c r="K16" s="33" t="n"/>
+      <c r="L16" s="33" t="n"/>
       <c r="N16" s="34">
         <f>IF($A16="",NA(),IF(C16&gt;0,D16/C16,0))</f>
         <v/>
@@ -3598,46 +3140,16 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>18:35:00</t>
-        </is>
-      </c>
-      <c r="C17" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D17" s="33" t="n">
-        <v>306849</v>
-      </c>
-      <c r="E17" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F17" s="33" t="n">
-        <v>101695107</v>
-      </c>
-      <c r="G17" s="33" t="n">
-        <v>101542564</v>
-      </c>
-      <c r="H17" s="33" t="n">
-        <v>80218626</v>
-      </c>
-      <c r="I17" s="33" t="n">
-        <v>80218626</v>
-      </c>
-      <c r="J17" s="33" t="n">
-        <v>76608788</v>
-      </c>
-      <c r="K17" s="33" t="n">
-        <v>39063102</v>
-      </c>
-      <c r="L17" s="33" t="n">
-        <v>37545686</v>
-      </c>
+      <c r="C17" s="33" t="n"/>
+      <c r="D17" s="33" t="n"/>
+      <c r="E17" s="33" t="n"/>
+      <c r="F17" s="33" t="n"/>
+      <c r="G17" s="33" t="n"/>
+      <c r="H17" s="33" t="n"/>
+      <c r="I17" s="33" t="n"/>
+      <c r="J17" s="33" t="n"/>
+      <c r="K17" s="33" t="n"/>
+      <c r="L17" s="33" t="n"/>
       <c r="N17" s="34">
         <f>IF($A17="",NA(),IF(C17&gt;0,D17/C17,0))</f>
         <v/>
@@ -3672,46 +3184,16 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>18:41:00</t>
-        </is>
-      </c>
-      <c r="C18" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D18" s="33" t="n">
-        <v>330452</v>
-      </c>
-      <c r="E18" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F18" s="33" t="n">
-        <v>109517808</v>
-      </c>
-      <c r="G18" s="33" t="n">
-        <v>109353531</v>
-      </c>
-      <c r="H18" s="33" t="n">
-        <v>86389289</v>
-      </c>
-      <c r="I18" s="33" t="n">
-        <v>86389289</v>
-      </c>
-      <c r="J18" s="33" t="n">
-        <v>82501771</v>
-      </c>
-      <c r="K18" s="33" t="n">
-        <v>41866992</v>
-      </c>
-      <c r="L18" s="33" t="n">
-        <v>40634779</v>
-      </c>
+      <c r="C18" s="33" t="n"/>
+      <c r="D18" s="33" t="n"/>
+      <c r="E18" s="33" t="n"/>
+      <c r="F18" s="33" t="n"/>
+      <c r="G18" s="33" t="n"/>
+      <c r="H18" s="33" t="n"/>
+      <c r="I18" s="33" t="n"/>
+      <c r="J18" s="33" t="n"/>
+      <c r="K18" s="33" t="n"/>
+      <c r="L18" s="33" t="n"/>
       <c r="N18" s="34">
         <f>IF($A18="",NA(),IF(C18&gt;0,D18/C18,0))</f>
         <v/>
@@ -3746,46 +3228,16 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>18:47:00</t>
-        </is>
-      </c>
-      <c r="C19" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D19" s="33" t="n">
-        <v>349336</v>
-      </c>
-      <c r="E19" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F19" s="33" t="n">
-        <v>115775968</v>
-      </c>
-      <c r="G19" s="33" t="n">
-        <v>115602304</v>
-      </c>
-      <c r="H19" s="33" t="n">
-        <v>91325820</v>
-      </c>
-      <c r="I19" s="33" t="n">
-        <v>91325820</v>
-      </c>
-      <c r="J19" s="33" t="n">
-        <v>87216158</v>
-      </c>
-      <c r="K19" s="33" t="n">
-        <v>44086665</v>
-      </c>
-      <c r="L19" s="33" t="n">
-        <v>43129493</v>
-      </c>
+      <c r="C19" s="33" t="n"/>
+      <c r="D19" s="33" t="n"/>
+      <c r="E19" s="33" t="n"/>
+      <c r="F19" s="33" t="n"/>
+      <c r="G19" s="33" t="n"/>
+      <c r="H19" s="33" t="n"/>
+      <c r="I19" s="33" t="n"/>
+      <c r="J19" s="33" t="n"/>
+      <c r="K19" s="33" t="n"/>
+      <c r="L19" s="33" t="n"/>
       <c r="N19" s="34">
         <f>IF($A19="",NA(),IF(C19&gt;0,D19/C19,0))</f>
         <v/>
@@ -3820,46 +3272,16 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>18:53:00</t>
-        </is>
-      </c>
-      <c r="C20" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D20" s="33" t="n">
-        <v>368218</v>
-      </c>
-      <c r="E20" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F20" s="33" t="n">
-        <v>122034129</v>
-      </c>
-      <c r="G20" s="33" t="n">
-        <v>121851078</v>
-      </c>
-      <c r="H20" s="33" t="n">
-        <v>96262352</v>
-      </c>
-      <c r="I20" s="33" t="n">
-        <v>96262352</v>
-      </c>
-      <c r="J20" s="33" t="n">
-        <v>91930546</v>
-      </c>
-      <c r="K20" s="33" t="n">
-        <v>46285188</v>
-      </c>
-      <c r="L20" s="33" t="n">
-        <v>45645358</v>
-      </c>
+      <c r="C20" s="33" t="n"/>
+      <c r="D20" s="33" t="n"/>
+      <c r="E20" s="33" t="n"/>
+      <c r="F20" s="33" t="n"/>
+      <c r="G20" s="33" t="n"/>
+      <c r="H20" s="33" t="n"/>
+      <c r="I20" s="33" t="n"/>
+      <c r="J20" s="33" t="n"/>
+      <c r="K20" s="33" t="n"/>
+      <c r="L20" s="33" t="n"/>
       <c r="N20" s="34">
         <f>IF($A20="",NA(),IF(C20&gt;0,D20/C20,0))</f>
         <v/>
@@ -3894,46 +3316,16 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>18:59:00</t>
-        </is>
-      </c>
-      <c r="C21" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D21" s="33" t="n">
-        <v>387102</v>
-      </c>
-      <c r="E21" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F21" s="33" t="n">
-        <v>128292289</v>
-      </c>
-      <c r="G21" s="33" t="n">
-        <v>128099851</v>
-      </c>
-      <c r="H21" s="33" t="n">
-        <v>101198882</v>
-      </c>
-      <c r="I21" s="33" t="n">
-        <v>101198882</v>
-      </c>
-      <c r="J21" s="33" t="n">
-        <v>96644932</v>
-      </c>
-      <c r="K21" s="33" t="n">
-        <v>48462278</v>
-      </c>
-      <c r="L21" s="33" t="n">
-        <v>48182654</v>
-      </c>
+      <c r="C21" s="33" t="n"/>
+      <c r="D21" s="33" t="n"/>
+      <c r="E21" s="33" t="n"/>
+      <c r="F21" s="33" t="n"/>
+      <c r="G21" s="33" t="n"/>
+      <c r="H21" s="33" t="n"/>
+      <c r="I21" s="33" t="n"/>
+      <c r="J21" s="33" t="n"/>
+      <c r="K21" s="33" t="n"/>
+      <c r="L21" s="33" t="n"/>
       <c r="N21" s="34">
         <f>IF($A21="",NA(),IF(C21&gt;0,D21/C21,0))</f>
         <v/>
@@ -3968,46 +3360,16 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>19:05:00</t>
-        </is>
-      </c>
-      <c r="C22" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D22" s="33" t="n">
-        <v>401264</v>
-      </c>
-      <c r="E22" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F22" s="33" t="n">
-        <v>132985909</v>
-      </c>
-      <c r="G22" s="33" t="n">
-        <v>132786430</v>
-      </c>
-      <c r="H22" s="33" t="n">
-        <v>104901280</v>
-      </c>
-      <c r="I22" s="33" t="n">
-        <v>104901280</v>
-      </c>
-      <c r="J22" s="33" t="n">
-        <v>100180722</v>
-      </c>
-      <c r="K22" s="33" t="n">
-        <v>50080869</v>
-      </c>
-      <c r="L22" s="33" t="n">
-        <v>50099853</v>
-      </c>
+      <c r="C22" s="33" t="n"/>
+      <c r="D22" s="33" t="n"/>
+      <c r="E22" s="33" t="n"/>
+      <c r="F22" s="33" t="n"/>
+      <c r="G22" s="33" t="n"/>
+      <c r="H22" s="33" t="n"/>
+      <c r="I22" s="33" t="n"/>
+      <c r="J22" s="33" t="n"/>
+      <c r="K22" s="33" t="n"/>
+      <c r="L22" s="33" t="n"/>
       <c r="N22" s="34">
         <f>IF($A22="",NA(),IF(C22&gt;0,D22/C22,0))</f>
         <v/>
@@ -4042,46 +3404,16 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>19:11:00</t>
-        </is>
-      </c>
-      <c r="C23" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D23" s="33" t="n">
-        <v>415426</v>
-      </c>
-      <c r="E23" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F23" s="33" t="n">
-        <v>137679530</v>
-      </c>
-      <c r="G23" s="33" t="n">
-        <v>137473011</v>
-      </c>
-      <c r="H23" s="33" t="n">
-        <v>108603679</v>
-      </c>
-      <c r="I23" s="33" t="n">
-        <v>108603679</v>
-      </c>
-      <c r="J23" s="33" t="n">
-        <v>103716513</v>
-      </c>
-      <c r="K23" s="33" t="n">
-        <v>51687143</v>
-      </c>
-      <c r="L23" s="33" t="n">
-        <v>52029370</v>
-      </c>
+      <c r="C23" s="33" t="n"/>
+      <c r="D23" s="33" t="n"/>
+      <c r="E23" s="33" t="n"/>
+      <c r="F23" s="33" t="n"/>
+      <c r="G23" s="33" t="n"/>
+      <c r="H23" s="33" t="n"/>
+      <c r="I23" s="33" t="n"/>
+      <c r="J23" s="33" t="n"/>
+      <c r="K23" s="33" t="n"/>
+      <c r="L23" s="33" t="n"/>
       <c r="N23" s="34">
         <f>IF($A23="",NA(),IF(C23&gt;0,D23/C23,0))</f>
         <v/>
@@ -4116,46 +3448,16 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>19:17:00</t>
-        </is>
-      </c>
-      <c r="C24" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D24" s="33" t="n">
-        <v>427228</v>
-      </c>
-      <c r="E24" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F24" s="33" t="n">
-        <v>141590880</v>
-      </c>
-      <c r="G24" s="33" t="n">
-        <v>141378494</v>
-      </c>
-      <c r="H24" s="33" t="n">
-        <v>111689010</v>
-      </c>
-      <c r="I24" s="33" t="n">
-        <v>111689010</v>
-      </c>
-      <c r="J24" s="33" t="n">
-        <v>106663005</v>
-      </c>
-      <c r="K24" s="33" t="n">
-        <v>53016218</v>
-      </c>
-      <c r="L24" s="33" t="n">
-        <v>53646787</v>
-      </c>
+      <c r="C24" s="33" t="n"/>
+      <c r="D24" s="33" t="n"/>
+      <c r="E24" s="33" t="n"/>
+      <c r="F24" s="33" t="n"/>
+      <c r="G24" s="33" t="n"/>
+      <c r="H24" s="33" t="n"/>
+      <c r="I24" s="33" t="n"/>
+      <c r="J24" s="33" t="n"/>
+      <c r="K24" s="33" t="n"/>
+      <c r="L24" s="33" t="n"/>
       <c r="N24" s="34">
         <f>IF($A24="",NA(),IF(C24&gt;0,D24/C24,0))</f>
         <v/>
@@ -4190,46 +3492,16 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>19:23:00</t>
-        </is>
-      </c>
-      <c r="C25" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D25" s="33" t="n">
-        <v>436669</v>
-      </c>
-      <c r="E25" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F25" s="33" t="n">
-        <v>144719960</v>
-      </c>
-      <c r="G25" s="33" t="n">
-        <v>144502880</v>
-      </c>
-      <c r="H25" s="33" t="n">
-        <v>114157275</v>
-      </c>
-      <c r="I25" s="33" t="n">
-        <v>114157275</v>
-      </c>
-      <c r="J25" s="33" t="n">
-        <v>109020198</v>
-      </c>
-      <c r="K25" s="33" t="n">
-        <v>54073225</v>
-      </c>
-      <c r="L25" s="33" t="n">
-        <v>54946973</v>
-      </c>
+      <c r="C25" s="33" t="n"/>
+      <c r="D25" s="33" t="n"/>
+      <c r="E25" s="33" t="n"/>
+      <c r="F25" s="33" t="n"/>
+      <c r="G25" s="33" t="n"/>
+      <c r="H25" s="33" t="n"/>
+      <c r="I25" s="33" t="n"/>
+      <c r="J25" s="33" t="n"/>
+      <c r="K25" s="33" t="n"/>
+      <c r="L25" s="33" t="n"/>
       <c r="N25" s="34">
         <f>IF($A25="",NA(),IF(C25&gt;0,D25/C25,0))</f>
         <v/>
@@ -4264,46 +3536,16 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>25/10/2026</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>19:29:00</t>
-        </is>
-      </c>
-      <c r="C26" s="33" t="n">
-        <v>472075</v>
-      </c>
-      <c r="D26" s="33" t="n">
-        <v>443750</v>
-      </c>
-      <c r="E26" s="33" t="n">
-        <v>156454011</v>
-      </c>
-      <c r="F26" s="33" t="n">
-        <v>147066770</v>
-      </c>
-      <c r="G26" s="33" t="n">
-        <v>146846170</v>
-      </c>
-      <c r="H26" s="33" t="n">
-        <v>116008474</v>
-      </c>
-      <c r="I26" s="33" t="n">
-        <v>116008474</v>
-      </c>
-      <c r="J26" s="33" t="n">
-        <v>110788093</v>
-      </c>
-      <c r="K26" s="33" t="n">
-        <v>54862312</v>
-      </c>
-      <c r="L26" s="33" t="n">
-        <v>55925781</v>
-      </c>
+      <c r="C26" s="33" t="n"/>
+      <c r="D26" s="33" t="n"/>
+      <c r="E26" s="33" t="n"/>
+      <c r="F26" s="33" t="n"/>
+      <c r="G26" s="33" t="n"/>
+      <c r="H26" s="33" t="n"/>
+      <c r="I26" s="33" t="n"/>
+      <c r="J26" s="33" t="n"/>
+      <c r="K26" s="33" t="n"/>
+      <c r="L26" s="33" t="n"/>
       <c r="N26" s="34">
         <f>IF($A26="",NA(),IF(C26&gt;0,D26/C26,0))</f>
         <v/>
@@ -47530,7 +46772,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>•</t>
@@ -47538,7 +46780,7 @@
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>Apague os dados de demonstração: Dados!A2:B40 e Dados!E2:K20 (só os valores) e Histórico!A2:L1001.</t>
+          <t>Caminho mais simples: o painel web da pasta painel-ao-vivo (dois cliques, já conectado). Esta planilha é a alternativa para quem quer os números no Excel ou no Google Planilhas.</t>
         </is>
       </c>
     </row>
@@ -47569,7 +46811,7 @@
       </c>
       <c r="B8" s="25" t="inlineStr">
         <is>
-          <t>Apague também os CABEÇALHOS: Dados!A1:B1, Dados!E1:K1 e Histórico!A1:L1 (as consultas recriam).</t>
+          <t>Apague (tecla Delete) Dados!A1:B40, Dados!E1:K20 e Histórico!A1:L1: as consultas recriam esses dados e cabeçalhos.</t>
         </is>
       </c>
     </row>

</xml_diff>